<commit_message>
Adiciona lançamento: Itabus Rome-Bari (02/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +92,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -457,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -491,6 +493,31 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Classe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Itabus Rome-Bari Acheminement guide</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>hors séjour</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Rosso Pomodoro-dîner guide (03/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,31 @@
         <v>22.99</v>
       </c>
       <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>hors séjour</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Rosso Pomodoro-dîner guide</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>hors séjour</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: Il Fortino-Diner Guide (04/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -541,6 +541,31 @@
         <v>28</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>hors séjour</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Il Fortino-Diner Guide</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>hors séjour</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: Maiora-déjeuner du guide (04/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -566,6 +566,31 @@
         <v>14.5</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>hors séjour</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Maiora-déjeuner du guide</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>hors séjour</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: train bari-polignano (07/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -593,6 +593,31 @@
       <c r="E5" s="6" t="inlineStr">
         <is>
           <t>hors séjour</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>train bari-polignano</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: bus locorotondo-albertobello (08/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -616,6 +616,31 @@
         <v>44.8</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>bus locorotondo-albertobello</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>transport</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: bus albertobello-martina (09/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,31 @@
         <v>20.8</v>
       </c>
       <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>bus albertobello-martina</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>transport</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: train martina cisternino (09/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -666,6 +666,31 @@
         <v>20.8</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>train martina cisternino</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>transport</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: train ostuni lecce (10/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -691,6 +691,31 @@
         <v>20.8</v>
       </c>
       <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>train ostuni lecce</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>transport</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: train lecce bari (11/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -716,6 +716,31 @@
         <v>100.8</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>train lecce bari</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>190.4</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>transport</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: maiora (06/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,31 @@
       <c r="E11" s="6" t="inlineStr">
         <is>
           <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>maiora</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>165.68</v>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: pizzeria enzo e ciro (06/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -768,6 +768,31 @@
       <c r="E12" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>pizzeria enzo e ciro</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>repas accompagnateur</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: fruta delária (07/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -793,6 +793,31 @@
       <c r="E13" s="6" t="inlineStr">
         <is>
           <t>repas accompagnateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>fruta delária</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>picnic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Supermercado Alberobello (07/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -816,6 +816,31 @@
         <v>23</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>picnic</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Supermercado Alberobello</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>picnic</t>
         </is>

</xml_diff>

<commit_message>
Padroniza grafia de Classe "pique nique" e documenta a convenção
Corrige linhas 14 e 15 (estavam como "picnic") para manter a mesma
grafia usada na linha 12.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -817,7 +817,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>picnic</t>
+          <t>pique nique</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>picnic</t>
+          <t>pique nique</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Supermercado Alberobello (08/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -841,6 +841,31 @@
         <v>71.2</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Supermercado Alberobello</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: bus albertobello-martina (08/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -868,6 +868,31 @@
       <c r="E16" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>bus albertobello-martina</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>transport</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Panifício (09/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -918,6 +918,31 @@
       <c r="E18" s="6" t="inlineStr">
         <is>
           <t>transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Panifício</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Alimentari (09/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -941,6 +941,31 @@
         <v>2.45</v>
       </c>
       <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Alimentari</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>45.88</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamentos: bottega italiana e il delfino (10/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -966,6 +966,56 @@
         <v>45.88</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>bottega italiana</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>il delfino</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>98.31999999999999</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
         </is>

</xml_diff>

<commit_message>
Adiciona lançamento: mudo (11/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1018,6 +1018,31 @@
       <c r="E22" s="6" t="inlineStr">
         <is>
           <t>pique nique</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>mudo</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>visitas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lançamento: Rapa it repas baia Orte (11/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,31 @@
       <c r="E23" s="6" t="inlineStr">
         <is>
           <t>visitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Rapa it repas baia Orte</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>270</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>pique nique</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renomeia classe "pique nique" para "FRAIS PIQUE-NIQUES"
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -767,7 +767,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>pique nique</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renomeia classe "transport" para "FRAIS TRANSPORT DU GROUPE (tickets de bus,…)"
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>transport</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renomeia classe "hors séjour" para "NOTE DE FRAIS HORS SEJOUR"
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>hors séjour</t>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>hors séjour</t>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>hors séjour</t>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>hors séjour</t>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorganiza planilha: lançamentos agrupados por classe com subtotais
Linhas agrupadas por Classe (ordenadas por data dentro de cada grupo),
com linha de subtotal (fórmula SUM) por classe e TOTAL GERAL no fim.
Reorganização pontual: novos lançamentos voltam a ser adicionados no
fim da lista via scripts/add_lancamento.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -44,7 +44,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -56,8 +56,23 @@
         <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00808080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00203864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -79,11 +94,56 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -94,6 +154,14 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -497,39 +565,25 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Itabus Rome-Bari Acheminement guide</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>22.99</v>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Rosso Pomodoro-dîner guide</t>
+          <t>Itabus Rome-Bari Acheminement guide</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -538,7 +592,7 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>28</v>
+        <v>22.99</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
@@ -549,12 +603,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Il Fortino-Diner Guide</t>
+          <t>Rosso Pomodoro-dîner guide</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -563,7 +617,7 @@
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>14.5</v>
+        <v>28</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
@@ -579,7 +633,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Maiora-déjeuner du guide</t>
+          <t>Il Fortino-Diner Guide</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -588,7 +642,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>9.92</v>
+        <v>14.5</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -599,12 +653,12 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>train bari-polignano</t>
+          <t>Maiora-déjeuner du guide</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -613,98 +667,55 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>44.8</v>
+        <v>9.92</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="12">
+        <f>SUM(D3:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="11" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n"/>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>bus locorotondo-albertobello</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>bus albertobello-martina</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>train martina cisternino</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>train ostuni lecce</t>
+          <t>train bari-polignano</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -713,7 +724,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>100.8</v>
+        <v>44.8</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -724,12 +735,12 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>train lecce bari</t>
+          <t>bus locorotondo-albertobello</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -738,7 +749,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>190.4</v>
+        <v>20.8</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
@@ -749,12 +760,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>06/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>maiora</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -763,23 +774,23 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>165.68</v>
+        <v>2.6</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>06/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>pizzeria enzo e ciro</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -788,23 +799,23 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>31</v>
+        <v>18.2</v>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>fruta delária</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -813,23 +824,23 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>23</v>
+        <v>20.8</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Supermercado Alberobello</t>
+          <t>train martina cisternino</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -838,23 +849,23 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>71.2</v>
+        <v>20.8</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Supermercado Alberobello</t>
+          <t>train ostuni lecce</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -863,23 +874,23 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>3</v>
+        <v>100.8</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>bus albertobello-martina</t>
+          <t>train lecce bari</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -888,7 +899,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2.6</v>
+        <v>190.4</v>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
@@ -897,89 +908,46 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>bus albertobello-martina</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="12">
+        <f>SUM(D10:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Panifício</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Alimentari</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>45.88</v>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>bottega italiana</t>
+          <t>maiora</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -988,7 +956,7 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>15</v>
+        <v>165.68</v>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
@@ -999,12 +967,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>il delfino</t>
+          <t>fruta delária</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1013,7 +981,7 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>98.31999999999999</v>
+        <v>23</v>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
@@ -1024,12 +992,12 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>mudo</t>
+          <t>Supermercado Alberobello</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1038,40 +1006,301 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>30</v>
+        <v>71.2</v>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>FRAIS VISITES</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Supermercado Alberobello</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Panifício</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Alimentari</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>45.88</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>bottega italiana</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>il delfino</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>98.31999999999999</v>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Rapa it repas baia Orte</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="n">
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="12">
+        <f>SUM(D21:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="11" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>06/09/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>pizzeria enzo e ciro</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="12">
+        <f>SUM(D33:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="10" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>mudo</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="12">
+        <f>SUM(D37:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="15">
+        <f>D7+D18+D30+D34+D38</f>
+        <v/>
+      </c>
+      <c r="E40" s="14" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reordena classes na planilha agrupada
Ordem: FRAIS PIQUE-NIQUES, FRAIS TAXES DE SEJOUR REPAS Accompagnateur,
FRAIS VISITES, FRAIS TRANSPORT DU GROUPE, NOTE DE FRAIS HORS SEJOUR.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
       <c r="B2" s="9" t="n"/>
@@ -578,12 +578,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>02/09/2026</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Itabus Rome-Bari Acheminement guide</t>
+          <t>maiora</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -592,23 +592,23 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>22.99</v>
+        <v>165.68</v>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Rosso Pomodoro-dîner guide</t>
+          <t>fruta delária</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -617,23 +617,23 @@
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Il Fortino-Diner Guide</t>
+          <t>Supermercado Alberobello</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -642,23 +642,23 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>14.5</v>
+        <v>71.2</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Maiora-déjeuner du guide</t>
+          <t>Supermercado Alberobello</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -667,55 +667,98 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>9.92</v>
+        <v>3</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12">
-        <f>SUM(D3:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="11" t="n"/>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Panifício</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n"/>
-      <c r="B8" s="13" t="n"/>
-      <c r="C8" s="13" t="n"/>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="13" t="n"/>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Alimentari</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>45.88</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="10" t="n"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>bottega italiana</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>train bari-polignano</t>
+          <t>il delfino</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -724,23 +767,23 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>44.8</v>
+        <v>98.31999999999999</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>bus locorotondo-albertobello</t>
+          <t>Rapa it repas baia Orte</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -749,98 +792,55 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>20.8</v>
+        <v>270</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+          <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>bus albertobello-martina</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="12">
+        <f>SUM(D3:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>bus albertobello-martina</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="A13" s="13" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>09/09/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>bus albertobello-martina</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>train martina cisternino</t>
+          <t>pizzeria enzo e ciro</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -849,145 +849,102 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>20.8</v>
+        <v>31</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="12">
+        <f>SUM(D15:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="10" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>mudo</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="12">
+        <f>SUM(D19:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>10/09/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>train ostuni lecce</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>100.8</v>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>train lecce bari</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>190.4</v>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="12">
-        <f>SUM(D10:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="11" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="13" t="n"/>
-      <c r="C19" s="13" t="n"/>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="10" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>06/09/2026</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>maiora</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>165.68</v>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>fruta delária</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -997,7 +954,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Supermercado Alberobello</t>
+          <t>train bari-polignano</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1006,11 +963,11 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>71.2</v>
+        <v>44.8</v>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
@@ -1022,7 +979,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Supermercado Alberobello</t>
+          <t>bus locorotondo-albertobello</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1031,23 +988,23 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>3</v>
+        <v>20.8</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Panifício</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1056,23 +1013,23 @@
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>2.45</v>
+        <v>2.6</v>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Alimentari</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1081,23 +1038,23 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>45.88</v>
+        <v>18.2</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>bottega italiana</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1106,23 +1063,23 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>15</v>
+        <v>20.8</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>il delfino</t>
+          <t>train martina cisternino</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1131,123 +1088,180 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>98.31999999999999</v>
+        <v>20.8</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>FRAIS PIQUE-NIQUES</t>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>train ostuni lecce</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Rapa it repas baia Orte</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>270</v>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>train lecce bari</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>190.4</v>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="12">
-        <f>SUM(D21:D29)</f>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="12">
+        <f>SUM(D23:D30)</f>
         <v/>
       </c>
-      <c r="E30" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="10" t="n"/>
+      <c r="A32" s="13" t="n"/>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>06/09/2026</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>pizzeria enzo e ciro</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D33" s="7" t="n">
-        <v>31</v>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
-        </is>
-      </c>
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="10" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="11" t="n"/>
-      <c r="D34" s="12">
-        <f>SUM(D33:D33)</f>
-        <v/>
-      </c>
-      <c r="E34" s="11" t="n"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Itabus Rome-Bari Acheminement guide</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Rosso Pomodoro-dîner guide</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>FRAIS VISITES</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n"/>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="10" t="n"/>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Il Fortino-Diner Guide</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>mudo</t>
+          <t>Maiora-déjeuner du guide</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -1256,11 +1270,11 @@
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>30</v>
+        <v>9.92</v>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>FRAIS VISITES</t>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
@@ -1273,10 +1287,17 @@
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="11" t="n"/>
       <c r="D38" s="12">
-        <f>SUM(D37:D37)</f>
+        <f>SUM(D34:D37)</f>
         <v/>
       </c>
       <c r="E38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="n"/>
+      <c r="B39" s="13" t="n"/>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="13" t="n"/>
+      <c r="E39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
@@ -1287,19 +1308,19 @@
       <c r="B40" s="9" t="n"/>
       <c r="C40" s="10" t="n"/>
       <c r="D40" s="15">
-        <f>D7+D18+D30+D34+D38</f>
+        <f>D12+D16+D20+D31+D38</f>
         <v/>
       </c>
       <c r="E40" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona título "Séjour Pouilles du Sud" no topo da planilha
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,11 @@
     </font>
     <font>
       <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="6">
@@ -143,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +167,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -537,78 +543,60 @@
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Séjour Pouilles du Sud - 06/09/2026 à 12/09/2026 - Acc. Felipe DINIZ PAIVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>DATES (JJ/MM/AAAA)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>DESIGNATION</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>N° du justificatif</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>MONTANT EN EUROS</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Classe</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="10" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>06/09/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>maiora</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>165.68</v>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS PIQUE-NIQUES</t>
-        </is>
-      </c>
+      <c r="B3" s="9" t="n"/>
+      <c r="C3" s="9" t="n"/>
+      <c r="D3" s="9" t="n"/>
+      <c r="E3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>07/09/2026</t>
+          <t>06/09/2026</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>fruta delária</t>
+          <t>maiora</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -617,7 +605,7 @@
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>23</v>
+        <v>165.68</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
@@ -633,7 +621,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Supermercado Alberobello</t>
+          <t>fruta delária</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -642,7 +630,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>71.2</v>
+        <v>23</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -653,7 +641,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -667,7 +655,7 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>3</v>
+        <v>71.2</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -678,12 +666,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Panifício</t>
+          <t>Supermercado Alberobello</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -692,7 +680,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2.45</v>
+        <v>3</v>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
@@ -708,7 +696,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Alimentari</t>
+          <t>Panifício</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -717,7 +705,7 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>45.88</v>
+        <v>2.45</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
@@ -728,12 +716,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>bottega italiana</t>
+          <t>Alimentari</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -742,7 +730,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>15</v>
+        <v>45.88</v>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
@@ -758,7 +746,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>il delfino</t>
+          <t>bottega italiana</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -767,7 +755,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>98.31999999999999</v>
+        <v>15</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -778,208 +766,208 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>il delfino</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>98.31999999999999</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Rapa it repas baia Orte</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
         <v>270</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>FRAIS PIQUE-NIQUES</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="12">
-        <f>SUM(D3:D11)</f>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="12">
+        <f>SUM(D4:D12)</f>
         <v/>
       </c>
-      <c r="E12" s="11" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
+      <c r="E13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="13" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>06/09/2026</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>pizzeria enzo e ciro</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="n">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
         <v>31</v>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="12">
-        <f>SUM(D15:D15)</f>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="12">
+        <f>SUM(D16:D16)</f>
         <v/>
       </c>
-      <c r="E16" s="11" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="13" t="n"/>
+      <c r="E17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>FRAIS VISITES</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="10" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>mudo</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>FRAIS VISITES</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="12">
-        <f>SUM(D19:D19)</f>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="12">
+        <f>SUM(D20:D20)</f>
         <v/>
       </c>
-      <c r="E20" s="11" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="13" t="n"/>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
+      <c r="E21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>train bari-polignano</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
-        </is>
-      </c>
+      <c r="B23" s="9" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>07/09/2026</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>bus locorotondo-albertobello</t>
+          <t>train bari-polignano</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -988,7 +976,7 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>20.8</v>
+        <v>44.8</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
@@ -1004,7 +992,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>bus albertobello-martina</t>
+          <t>bus locorotondo-albertobello</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1013,7 +1001,7 @@
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>2.6</v>
+        <v>20.8</v>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
@@ -1038,7 +1026,7 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>18.2</v>
+        <v>2.6</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
@@ -1049,7 +1037,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>09/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -1063,7 +1051,7 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>20.8</v>
+        <v>18.2</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
@@ -1079,7 +1067,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>train martina cisternino</t>
+          <t>bus albertobello-martina</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1099,12 +1087,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>10/09/2026</t>
+          <t>09/09/2026</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>train ostuni lecce</t>
+          <t>train martina cisternino</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -1113,7 +1101,7 @@
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>100.8</v>
+        <v>20.8</v>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
@@ -1124,94 +1112,94 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>train ostuni lecce</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>train lecce bari</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="n">
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
         <v>190.4</v>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="12">
-        <f>SUM(D23:D30)</f>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="12">
+        <f>SUM(D24:D31)</f>
         <v/>
       </c>
-      <c r="E31" s="11" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="n"/>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
+      <c r="E32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="13" t="n"/>
+      <c r="B33" s="13" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="10" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Itabus Rome-Bari Acheminement guide</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="n">
-        <v>22.99</v>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
-        </is>
-      </c>
+      <c r="B34" s="9" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>03/09/2026</t>
+          <t>02/09/2026</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Rosso Pomodoro-dîner guide</t>
+          <t>Itabus Rome-Bari Acheminement guide</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -1220,7 +1208,7 @@
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>28</v>
+        <v>22.99</v>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
@@ -1231,12 +1219,12 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>03/09/2026</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Il Fortino-Diner Guide</t>
+          <t>Rosso Pomodoro-dîner guide</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -1245,7 +1233,7 @@
         </is>
       </c>
       <c r="D36" s="7" t="n">
-        <v>14.5</v>
+        <v>28</v>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
@@ -1261,66 +1249,92 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
+          <t>Il Fortino-Diner Guide</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
           <t>Maiora-déjeuner du guide</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="n">
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
         <v>9.92</v>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="B38" s="11" t="n"/>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="12">
-        <f>SUM(D34:D37)</f>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="12">
+        <f>SUM(D35:D38)</f>
         <v/>
       </c>
-      <c r="E38" s="11" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="n"/>
-      <c r="B39" s="13" t="n"/>
-      <c r="C39" s="13" t="n"/>
-      <c r="D39" s="13" t="n"/>
-      <c r="E39" s="13" t="n"/>
+      <c r="E39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="13" t="n"/>
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B40" s="9" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="15">
-        <f>D12+D16+D20+D31+D38</f>
+      <c r="B41" s="9" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="15">
+        <f>D13+D17+D21+D32+D39</f>
         <v/>
       </c>
-      <c r="E40" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A22:E22"/>
+  <mergeCells count="7">
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona adiantamento recebido e saldo a reembolsar
Abaixo do TOTAL GERAL: linha "Adiantamento recebido" (-900) e
"MONTANT À REMBOURSER" (fórmula = total geral + adiantamento).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00;(#,##0.00)"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -49,7 +51,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00203864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -148,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,6 +175,9 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -533,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1326,14 +1336,43 @@
       </c>
       <c r="E41" s="14" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Adiantamento recebido</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="18" t="n">
+        <v>-900</v>
+      </c>
+      <c r="E43" s="17" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>MONTANT À REMBOURSER</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="19">
+        <f>D41+D43</f>
+        <v/>
+      </c>
+      <c r="E44" s="14" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A43:C43"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Traduz textos estruturais da planilha para francês
Abas "Lançamentos"→"Dépenses" e "Legenda"→"Légende", "Subtotal"→
"Sous-total", "TOTAL GERAL"→"TOTAL GÉNÉRAL", "Adiantamento recebido"→
"Avance reçue", conteúdo da Légende traduzido. Conteúdo dos
lançamentos (DESIGNATION) não foi alterado, conforme pedido.
Atualiza scripts/add_lancamento.py e CLAUDE.md para o novo nome de
aba e localiza a próxima linha livre pelo último conteúdo real.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lançamentos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dépenses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Légende" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -826,7 +826,7 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Sous-total</t>
         </is>
       </c>
       <c r="B13" s="11" t="n"/>
@@ -883,7 +883,7 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Sous-total</t>
         </is>
       </c>
       <c r="B17" s="11" t="n"/>
@@ -940,7 +940,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Sous-total</t>
         </is>
       </c>
       <c r="B21" s="11" t="n"/>
@@ -1172,7 +1172,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Sous-total</t>
         </is>
       </c>
       <c r="B32" s="11" t="n"/>
@@ -1304,7 +1304,7 @@
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Sous-total</t>
         </is>
       </c>
       <c r="B39" s="11" t="n"/>
@@ -1325,7 +1325,7 @@
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>TOTAL GERAL</t>
+          <t>TOTAL GÉNÉRAL</t>
         </is>
       </c>
       <c r="B41" s="9" t="n"/>
@@ -1336,10 +1336,11 @@
       </c>
       <c r="E41" s="14" t="n"/>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>Adiantamento recebido</t>
+          <t>Avance reçue</t>
         </is>
       </c>
       <c r="B43" s="9" t="n"/>
@@ -1395,19 +1396,19 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Como preencher a planilha 'Lançamentos'</t>
+          <t>Comment remplir la feuille 'Dépenses'</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Coluna</t>
+          <t>Colonne</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Descrição</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1420,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Data do lançamento, sempre no formato dia/mês/ano.</t>
+          <t>Date de la dépense, toujours au format jour/mois/année.</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1432,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Descrição do gasto/lançamento.</t>
+          <t>Description de la dépense.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1444,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Número do comprovante/recibo correspondente.</t>
+          <t>Numéro du justificatif/reçu correspondant.</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1456,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Valor em euros, usando ponto ou vírgula decimal.</t>
+          <t>Montant en euros, avec un point ou une virgule décimale.</t>
         </is>
       </c>
     </row>
@@ -1467,14 +1468,14 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Classe/categoria contábil do lançamento.</t>
+          <t>Classe/catégorie comptable de la dépense.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Exemplo de linha (ordem exata das colunas):</t>
+          <t>Exemple de ligne (ordre exact des colonnes) :</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove aba Légende da planilha
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/lancamentos.xlsx
+++ b/planilha/lancamentos.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Dépenses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Légende" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1336,7 +1335,6 @@
       </c>
       <c r="E41" s="14" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
@@ -1378,133 +1376,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Comment remplir la feuille 'Dépenses'</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Colonne</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>DATES (JJ/MM/AAAA)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Date de la dépense, toujours au format jour/mois/année.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>DESIGNATION</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Description de la dépense.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>N° du justificatif</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Numéro du justificatif/reçu correspondant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>MONTANT EN EUROS</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Montant en euros, avec un point ou une virgule décimale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Classe</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Classe/catégorie comptable de la dépense.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Exemple de ligne (ordre exact des colonnes) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>05/09/2026</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Achat fournitures de bureau</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>F2026-0001</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Classe 2</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>